<commit_message>
Update: Threat Alert Report - 2026-07-27 14:09
</commit_message>
<xml_diff>
--- a/excel_routes/route_AHB_CAI_threats.xlsx
+++ b/excel_routes/route_AHB_CAI_threats.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODERED\LAB\Artifacts\outputs\run_generated_260726_at_14.46\reports\excel_routes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODERED\LAB\Artifacts\outputs\run_generated_270726_at_12.25\reports\excel_routes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D62FED-CEE5-48B2-88E4-5201F45D53F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C5EB9E-15C0-4B8A-8957-90975D4E0A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12972" yWindow="348" windowWidth="10068" windowHeight="10284" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Currency</t>
   </si>
   <si>
-    <t>30-JUL-26</t>
+    <t>29-JUL-26</t>
   </si>
   <si>
     <t>SM-444</t>
@@ -75,10 +75,10 @@
     <t>SAR</t>
   </si>
   <si>
-    <t>01-AUG-26</t>
-  </si>
-  <si>
-    <t>Air Arabia Egypt E5-514</t>
+    <t>03-AUG-26</t>
+  </si>
+  <si>
+    <t>Air Arabia Egypt E5-512</t>
   </si>
   <si>
     <t>HIGH</t>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>10-SEP-26</t>
-  </si>
-  <si>
-    <t>Air Arabia Egypt E5-512</t>
   </si>
   <si>
     <t>30-OCT-26</t>
@@ -563,13 +560,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="2">
-        <v>506</v>
+        <v>453</v>
       </c>
       <c r="E2" s="2">
-        <v>518</v>
+        <v>491</v>
       </c>
       <c r="F2" s="2">
-        <v>-12</v>
+        <v>-38</v>
       </c>
       <c r="G2" s="2">
         <v>30</v>
@@ -598,13 +595,13 @@
         <v>17</v>
       </c>
       <c r="D3" s="2">
-        <v>776</v>
+        <v>580</v>
       </c>
       <c r="E3" s="2">
-        <v>1640</v>
+        <v>2400</v>
       </c>
       <c r="F3" s="2">
-        <v>-864</v>
+        <v>-1820</v>
       </c>
       <c r="G3" s="2">
         <v>20</v>
@@ -633,13 +630,13 @@
         <v>13</v>
       </c>
       <c r="D4" s="2">
-        <v>550</v>
+        <v>571</v>
       </c>
       <c r="E4" s="2">
         <v>592</v>
       </c>
       <c r="F4" s="2">
-        <v>-42</v>
+        <v>-21</v>
       </c>
       <c r="G4" s="2">
         <v>30</v>
@@ -805,16 +802,16 @@
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D9" s="2">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E9" s="2">
         <v>626</v>
       </c>
       <c r="F9" s="2">
-        <v>-156</v>
+        <v>-158</v>
       </c>
       <c r="G9" s="2">
         <v>20</v>
@@ -834,22 +831,22 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D10" s="2">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E10" s="2">
         <v>2635</v>
       </c>
       <c r="F10" s="2">
-        <v>-2063</v>
+        <v>-2065</v>
       </c>
       <c r="G10" s="2">
         <v>20</v>

</xml_diff>